<commit_message>
Creation Eddy_Branch + ajout 4 animation deplacement + repos sur zombie + gerer distance joueur
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nouveau dossier\Projet1_Jeux_Video\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17A5164-0C44-4963-8492-4F30C520D43D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{802D5BE2-6B86-4943-B8DC-33257F5B259C}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7010" yWindow="1430" windowWidth="16030" windowHeight="12250" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="58">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
   <si>
     <t>Fonctionnalites</t>
   </si>
@@ -312,6 +312,9 @@
   </si>
   <si>
     <t>tout le monde</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Tous ont 4 animations de déplacement (une pour chaque direction).:ok pour zombie</t>
   </si>
 </sst>
 </file>
@@ -879,16 +882,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B5B6CB-DB26-432C-9FC7-91B77E13F469}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.1796875" customWidth="1"/>
-    <col min="2" max="2" width="106.453125" customWidth="1"/>
-    <col min="3" max="3" width="57.08984375" customWidth="1"/>
-    <col min="4" max="4" width="36.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="77.6328125" customWidth="1"/>
+    <col min="1" max="1" width="41.21875" customWidth="1"/>
+    <col min="2" max="2" width="106.44140625" customWidth="1"/>
+    <col min="3" max="3" width="57.109375" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="55.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -905,7 +908,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="323.39999999999998" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:5" ht="323.39999999999998" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -920,7 +923,7 @@
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" ht="314.5" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:5" ht="306" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -935,7 +938,7 @@
       </c>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -950,7 +953,7 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="59.4" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:5" ht="59.4" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -965,7 +968,7 @@
       </c>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="220.75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:5" ht="220.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="14" t="s">
         <v>12</v>
       </c>
@@ -980,7 +983,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" ht="36" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:5" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -995,7 +998,7 @@
       </c>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -1010,7 +1013,7 @@
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
@@ -1025,7 +1028,7 @@
       </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -1040,7 +1043,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" ht="112.5" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:5" ht="150" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
@@ -1048,14 +1051,16 @@
         <v>22</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="12" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+      <c r="E11" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A12" s="5" t="s">
         <v>23</v>
       </c>
@@ -1070,7 +1075,7 @@
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -1085,7 +1090,7 @@
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
@@ -1100,7 +1105,7 @@
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
       <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
@@ -1115,7 +1120,7 @@
       </c>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
       <c r="A16" s="6" t="s">
         <v>31</v>
       </c>
@@ -1130,7 +1135,7 @@
       </c>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:6" ht="36" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:6" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
@@ -1145,7 +1150,7 @@
       </c>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:6" ht="36" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>35</v>
       </c>
@@ -1160,7 +1165,7 @@
       </c>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="1:6" ht="36" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
@@ -1175,7 +1180,7 @@
       </c>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:6" ht="56" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:6" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -1190,7 +1195,7 @@
       </c>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:6" ht="74" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" ht="72" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -1205,7 +1210,7 @@
       </c>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:6" ht="55.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" ht="54" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
@@ -1225,7 +1230,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="82.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" ht="82.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
Correction petit bug avec mouvement.
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Nouveau dossier\Projet1_Jeux_Video\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DDJV\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F17A5164-0C44-4963-8492-4F30C520D43D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C87EA834-6DC1-459D-89A9-6B5ED08ED159}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="7010" yWindow="1430" windowWidth="16030" windowHeight="12250" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
@@ -45,19 +45,6 @@
     <t>Texte</t>
   </si>
   <si>
-    <t xml:space="preserve">Niveau
-Un seul niveau bien conçu est demandé. On doit prendre soin d’avoir un visuel varié et soigné composé de plusieurs couches d’images. 
-1) Arrière-plan sur lequel le joueur marche (exemple : composition de gazon ou de terre).
-2) Doodads d’arrière-plan : petits objets décoratifs : plantes, cailloux, fleurs, etc.
-a. Au moins 3 différents non animés et fixe.
-b. Au moins 1 différent animé par du vent variable : ed :windsystem
-3) Doodads d’avant-plan animé : on doit voir minimum 2 entités (Exemple : nuages et oiseaux) se promener de gauche à droite à des vitesse variables. Ils doivent être petits ou semi-transparent afin de ne pas nuire à la visibilité du jeu.
-La limites de mouvement est de 3x3 la largeur de la grosseur de caméra que vous choisirez. Si le joueur dépasse cette limite, il est éliminé immédiatement.
-Cependant, quand le joueur près du bord de la carte, le visuel doit être adéquat pour 4x4 la largeur de la caméra.
-Exemple de conception adéquate : Une île bordée par de l’eau. Un donjon entouré de pics, une cave entourée de bras animées, etc.
-</t>
-  </si>
-  <si>
     <t>Joueur</t>
   </si>
   <si>
@@ -194,6 +181,91 @@
 • Barre d’expérience dans le haut de l’écran ou au-dessus du joueur.</t>
   </si>
   <si>
+    <t>Eddy</t>
+  </si>
+  <si>
+    <t>Commentaires</t>
+  </si>
+  <si>
+    <t>En cours</t>
+  </si>
+  <si>
+    <t>Pas commencé</t>
+  </si>
+  <si>
+    <t>Antoine</t>
+  </si>
+  <si>
+    <t>Charlee</t>
+  </si>
+  <si>
+    <t>nb vies + vitesse</t>
+  </si>
+  <si>
+    <t>Paul</t>
+  </si>
+  <si>
+    <t>****</t>
+  </si>
+  <si>
+    <t>tout le monde</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Niveau
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Un seul niveau bien conçu est demandé. On doit prendre soin d’avoir un visuel varié et soigné composé de plusieurs couches d’images. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>1) Arrière-plan sur lequel le joueur marche (exemple : composition de gazon ou de terre).</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+2) Doodads d’arrière-plan : petits objets décoratifs : plantes, cailloux, fleurs, etc.
+a. Au moins 3 différents non animés et fixe.
+b. Au moins 1 différent animé par du vent variable : ed :windsystem
+3) Doodads d’avant-plan animé : on doit voir minimum 2 entités (Exemple : nuages et oiseaux) se promener de gauche à droite à des vitesse variables. Ils doivent être petits ou semi-transparent afin de ne pas nuire à la visibilité du jeu.
+La limites de mouvement est de 3x3 la largeur de la grosseur de caméra que vous choisirez. Si le joueur dépasse cette limite, il est éliminé immédiatement.
+Cependant, quand le joueur près du bord de la carte, le visuel doit être adéquat pour 4x4 la largeur de la caméra.
+Exemple de conception adéquate : Une île bordée par de l’eau. Un donjon entouré de pics, une cave entourée de bras animées, etc.
+</t>
+    </r>
+  </si>
+  <si>
     <r>
       <rPr>
         <b/>
@@ -215,10 +287,90 @@
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">
-Attachez une Camera2D au joueur. Le joueur a 5 points de vie et commencera la partie avec une seule arme au choix. Si le joueur sort de la carte, il est automatiquement éliminé.
-• Animation
-o Animation unique quand ne bouge pas.
-o 4 animations différentes pour les 4 directions. Trouvez un tween pour agrémenter le mouvement.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Attachez une Camera2D au joueur.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Le joueur a 5 points de vie et commencera la partie avec une seule arme au choix. Si le joueur sort de la carte, il est automatiquement éliminé.
+• </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Animation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Animation unique quand ne bouge pas.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+o </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>4 animations différentes pour les 4 directions.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Trouvez un tween pour agrémenter le mouvement.
 o Animation unique lors d’une blessure accompagnée d’un tween.
 o Pour l’élimination, réutilisez l’animation unique de quand il ne bouge pas mais accompagnez le tout d’un tween et coloriez le joueur en rouge.
 o Pour la victoire, réutilisez l’animation unique de quand il ne bouge pas mais accompagnez le tout d’un tween et coloriez le joueur en vert.
@@ -282,43 +434,13 @@
       <t xml:space="preserve">
 </t>
     </r>
-  </si>
-  <si>
-    <t>Eddy</t>
-  </si>
-  <si>
-    <t>Commentaires</t>
-  </si>
-  <si>
-    <t>En cours</t>
-  </si>
-  <si>
-    <t>Pas commencé</t>
-  </si>
-  <si>
-    <t>Antoine</t>
-  </si>
-  <si>
-    <t>Charlee</t>
-  </si>
-  <si>
-    <t>nb vies + vitesse</t>
-  </si>
-  <si>
-    <t>Paul</t>
-  </si>
-  <si>
-    <t>****</t>
-  </si>
-  <si>
-    <t>tout le monde</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -392,6 +514,13 @@
       <b/>
       <sz val="26"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="14"/>
+      <color theme="9"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -902,7 +1031,7 @@
         <v>1</v>
       </c>
       <c r="E1" s="19" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
     </row>
     <row r="2" spans="1:5" ht="323.39999999999998" customHeight="1" x14ac:dyDescent="0.5">
@@ -910,333 +1039,333 @@
         <v>3</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>5</v>
+        <v>56</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D2" s="15" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" ht="314.5" x14ac:dyDescent="0.5">
       <c r="A3" s="3" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B3" s="8" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="C3" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D3" s="16" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E3" s="1"/>
     </row>
     <row r="4" spans="1:5" ht="56" x14ac:dyDescent="0.5">
       <c r="A4" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="7" t="s">
-        <v>8</v>
-      </c>
       <c r="C4" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D4" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E4" s="2"/>
     </row>
     <row r="5" spans="1:5" ht="59.4" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A5" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>10</v>
-      </c>
       <c r="C5" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D5" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E5" s="1"/>
     </row>
     <row r="6" spans="1:5" ht="220.75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A6" s="14" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B6" s="7" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C6" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D6" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="1:5" ht="36" x14ac:dyDescent="0.5">
       <c r="A7" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B7" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="9" t="s">
-        <v>14</v>
-      </c>
       <c r="C7" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E7" s="1"/>
     </row>
     <row r="8" spans="1:5" ht="56" x14ac:dyDescent="0.5">
       <c r="A8" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B8" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="7" t="s">
-        <v>16</v>
-      </c>
       <c r="C8" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E8" s="2"/>
     </row>
     <row r="9" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>18</v>
-      </c>
       <c r="C9" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D9" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D9" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E9" s="1"/>
     </row>
     <row r="10" spans="1:5" ht="56" x14ac:dyDescent="0.5">
       <c r="A10" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B10" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B10" s="7" t="s">
-        <v>20</v>
-      </c>
       <c r="C10" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10" s="15" t="s">
         <v>51</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>53</v>
       </c>
       <c r="E10" s="2"/>
     </row>
     <row r="11" spans="1:5" ht="112.5" x14ac:dyDescent="0.6">
       <c r="A11" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B11" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>22</v>
-      </c>
       <c r="C11" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D11" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E11" s="1"/>
     </row>
     <row r="12" spans="1:5" ht="36" x14ac:dyDescent="0.6">
       <c r="A12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="B12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>24</v>
-      </c>
       <c r="C12" s="18" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D12" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E12" s="2"/>
     </row>
     <row r="13" spans="1:5" ht="36" x14ac:dyDescent="0.6">
       <c r="A13" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="9" t="s">
-        <v>26</v>
-      </c>
       <c r="C13" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D13" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E13" s="1"/>
     </row>
     <row r="14" spans="1:5" ht="36" x14ac:dyDescent="0.6">
       <c r="A14" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="7" t="s">
-        <v>28</v>
-      </c>
       <c r="C14" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D14" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E14" s="2"/>
     </row>
     <row r="15" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
       <c r="A15" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B15" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="10" t="s">
-        <v>30</v>
-      </c>
       <c r="C15" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D15" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E15" s="1"/>
     </row>
     <row r="16" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
       <c r="A16" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B16" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="12" t="s">
-        <v>32</v>
-      </c>
       <c r="C16" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D16" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E16" s="2"/>
     </row>
     <row r="17" spans="1:6" ht="36" x14ac:dyDescent="0.6">
       <c r="A17" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="B17" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B17" s="9" t="s">
-        <v>34</v>
-      </c>
       <c r="C17" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D17" s="20" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E17" s="1"/>
     </row>
     <row r="18" spans="1:6" ht="36" x14ac:dyDescent="0.5">
       <c r="A18" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B18" s="13" t="s">
         <v>35</v>
       </c>
-      <c r="B18" s="13" t="s">
-        <v>36</v>
-      </c>
       <c r="C18" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D18" s="17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E18" s="2"/>
     </row>
     <row r="19" spans="1:6" ht="36" x14ac:dyDescent="0.5">
       <c r="A19" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B19" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="B19" s="9" t="s">
-        <v>38</v>
-      </c>
       <c r="C19" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D19" s="16" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E19" s="1"/>
     </row>
     <row r="20" spans="1:6" ht="56" x14ac:dyDescent="0.5">
       <c r="A20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="B20" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="B20" s="7" t="s">
-        <v>40</v>
-      </c>
       <c r="C20" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D20" s="15" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E20" s="2"/>
     </row>
     <row r="21" spans="1:6" ht="74" x14ac:dyDescent="0.45">
       <c r="A21" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B21" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="B21" s="9" t="s">
-        <v>42</v>
-      </c>
       <c r="C21" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E21" s="9"/>
     </row>
     <row r="22" spans="1:6" ht="55.5" x14ac:dyDescent="0.45">
       <c r="A22" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B22" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="B22" s="7" t="s">
-        <v>44</v>
-      </c>
       <c r="C22" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E22" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" s="21" t="s">
         <v>54</v>
-      </c>
-      <c r="F22" s="21" t="s">
-        <v>56</v>
       </c>
     </row>
     <row r="23" spans="1:6" ht="82.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="B23" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>46</v>
-      </c>
       <c r="C23" s="18" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E23" s="9"/>
     </row>

</xml_diff>

<commit_message>
fix collisions entres enemis + bug defered crystal
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="21929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\DDJV\Projet\Projet1_Jeux_Video\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C325F0F8-0376-4F67-A099-A65F99BE273E}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0C2A6B-16B1-4D72-8BCC-30FD30F2677B}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="23260" windowHeight="13900" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -314,10 +314,10 @@
     <t>tout le monde</t>
   </si>
   <si>
-    <t xml:space="preserve"> Tous ont 4 animations de déplacement (une pour chaque direction).:ok pour zombie</t>
-  </si>
-  <si>
     <t>Terminé</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> </t>
   </si>
 </sst>
 </file>
@@ -894,16 +894,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B5B6CB-DB26-432C-9FC7-91B77E13F469}">
   <dimension ref="A1:F23"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="41.1796875" customWidth="1"/>
-    <col min="2" max="2" width="106.453125" customWidth="1"/>
-    <col min="3" max="3" width="57.08984375" customWidth="1"/>
-    <col min="4" max="4" width="36.08984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="77.6328125" customWidth="1"/>
+    <col min="1" max="1" width="41.21875" customWidth="1"/>
+    <col min="2" max="2" width="106.44140625" customWidth="1"/>
+    <col min="3" max="3" width="57.109375" customWidth="1"/>
+    <col min="4" max="4" width="36.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="77.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="55.75" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
@@ -920,7 +920,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="323.39999999999998" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="2" spans="1:5" ht="323.39999999999998" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
@@ -928,14 +928,14 @@
         <v>5</v>
       </c>
       <c r="C2" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D2" s="15" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="2"/>
     </row>
-    <row r="3" spans="1:5" ht="314.5" x14ac:dyDescent="0.5">
+    <row r="3" spans="1:5" ht="306" x14ac:dyDescent="0.4">
       <c r="A3" s="3" t="s">
         <v>6</v>
       </c>
@@ -950,7 +950,7 @@
       </c>
       <c r="E3" s="1"/>
     </row>
-    <row r="4" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="4" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
@@ -965,7 +965,7 @@
       </c>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="59.4" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="5" spans="1:5" ht="59.4" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A5" s="3" t="s">
         <v>9</v>
       </c>
@@ -980,7 +980,7 @@
       </c>
       <c r="E5" s="1"/>
     </row>
-    <row r="6" spans="1:5" ht="220.75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="6" spans="1:5" ht="220.8" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A6" s="14" t="s">
         <v>12</v>
       </c>
@@ -995,7 +995,7 @@
       </c>
       <c r="E6" s="2"/>
     </row>
-    <row r="7" spans="1:5" ht="36" x14ac:dyDescent="0.5">
+    <row r="7" spans="1:5" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A7" s="3" t="s">
         <v>13</v>
       </c>
@@ -1010,7 +1010,7 @@
       </c>
       <c r="E7" s="1"/>
     </row>
-    <row r="8" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="8" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A8" s="2" t="s">
         <v>15</v>
       </c>
@@ -1018,14 +1018,14 @@
         <v>16</v>
       </c>
       <c r="C8" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D8" s="15" t="s">
         <v>53</v>
       </c>
       <c r="E8" s="2"/>
     </row>
-    <row r="9" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="9" spans="1:5" ht="75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A9" s="4" t="s">
         <v>17</v>
       </c>
@@ -1040,7 +1040,7 @@
       </c>
       <c r="E9" s="1"/>
     </row>
-    <row r="10" spans="1:5" ht="56" x14ac:dyDescent="0.5">
+    <row r="10" spans="1:5" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A10" s="2" t="s">
         <v>19</v>
       </c>
@@ -1055,7 +1055,7 @@
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" ht="150" customHeight="1" x14ac:dyDescent="0.6">
+    <row r="11" spans="1:5" ht="150" customHeight="1" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
@@ -1063,16 +1063,16 @@
         <v>22</v>
       </c>
       <c r="C11" s="18" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="12" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A12" s="5" t="s">
         <v>23</v>
       </c>
@@ -1080,14 +1080,14 @@
         <v>24</v>
       </c>
       <c r="C12" s="18" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="D12" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E12" s="2"/>
     </row>
-    <row r="13" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+    <row r="13" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A13" s="3" t="s">
         <v>25</v>
       </c>
@@ -1095,14 +1095,14 @@
         <v>26</v>
       </c>
       <c r="C13" s="18" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D13" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E13" s="1"/>
     </row>
-    <row r="14" spans="1:5" ht="36" x14ac:dyDescent="0.6">
+    <row r="14" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A14" s="2" t="s">
         <v>27</v>
       </c>
@@ -1110,14 +1110,14 @@
         <v>28</v>
       </c>
       <c r="C14" s="18" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D14" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E14" s="2"/>
     </row>
-    <row r="15" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
+    <row r="15" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
       <c r="A15" s="4" t="s">
         <v>29</v>
       </c>
@@ -1125,14 +1125,14 @@
         <v>30</v>
       </c>
       <c r="C15" s="18" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="D15" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E15" s="1"/>
     </row>
-    <row r="16" spans="1:5" ht="38.5" x14ac:dyDescent="0.6">
+    <row r="16" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
       <c r="A16" s="6" t="s">
         <v>31</v>
       </c>
@@ -1140,14 +1140,14 @@
         <v>32</v>
       </c>
       <c r="C16" s="18" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D16" s="20" t="s">
         <v>48</v>
       </c>
       <c r="E16" s="2"/>
     </row>
-    <row r="17" spans="1:6" ht="36" x14ac:dyDescent="0.6">
+    <row r="17" spans="1:6" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A17" s="3" t="s">
         <v>33</v>
       </c>
@@ -1162,7 +1162,7 @@
       </c>
       <c r="E17" s="1"/>
     </row>
-    <row r="18" spans="1:6" ht="36" x14ac:dyDescent="0.5">
+    <row r="18" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A18" s="6" t="s">
         <v>35</v>
       </c>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="E18" s="2"/>
     </row>
-    <row r="19" spans="1:6" ht="36" x14ac:dyDescent="0.5">
+    <row r="19" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
       <c r="A19" s="3" t="s">
         <v>37</v>
       </c>
@@ -1192,7 +1192,7 @@
       </c>
       <c r="E19" s="1"/>
     </row>
-    <row r="20" spans="1:6" ht="56" x14ac:dyDescent="0.5">
+    <row r="20" spans="1:6" ht="54.6" x14ac:dyDescent="0.4">
       <c r="A20" s="2" t="s">
         <v>39</v>
       </c>
@@ -1200,14 +1200,14 @@
         <v>40</v>
       </c>
       <c r="C20" s="22" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D20" s="15" t="s">
         <v>55</v>
       </c>
       <c r="E20" s="2"/>
     </row>
-    <row r="21" spans="1:6" ht="74" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:6" ht="72" x14ac:dyDescent="0.35">
       <c r="A21" s="3" t="s">
         <v>41</v>
       </c>
@@ -1222,7 +1222,7 @@
       </c>
       <c r="E21" s="9"/>
     </row>
-    <row r="22" spans="1:6" ht="55.5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:6" ht="54" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>43</v>
       </c>
@@ -1242,7 +1242,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="82.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:6" ht="82.2" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="3" t="s">
         <v>45</v>
       </c>

</xml_diff>

<commit_message>
Ajout Boss+ ses parents spwan pres du joueurl
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Download\_Cours_Eddy\_prog_jv\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0C2A6B-16B1-4D72-8BCC-30FD30F2677B}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1D7B477-FE5A-4540-9336-C91C44C20E4A}" xr6:coauthVersionLast="44" xr6:coauthVersionMax="44" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
   <si>
     <t>Fonctionnalites</t>
   </si>
@@ -319,12 +319,15 @@
   <si>
     <t xml:space="preserve"> </t>
   </si>
+  <si>
+    <t>Faire des vauges de spawn progressif des enemis</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -373,13 +376,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="16"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="28"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -397,6 +393,22 @@
     <font>
       <b/>
       <sz val="26"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -491,7 +503,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -534,28 +546,34 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -893,7 +911,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B5B6CB-DB26-432C-9FC7-91B77E13F469}">
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F24"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="41.21875" customWidth="1"/>
@@ -904,19 +922,19 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="55.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+      <c r="A1" s="16" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19" t="s">
+      <c r="B1" s="16" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="19" t="s">
+      <c r="C1" s="16" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="19" t="s">
+      <c r="D1" s="16" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="19" t="s">
+      <c r="E1" s="16" t="s">
         <v>49</v>
       </c>
     </row>
@@ -927,10 +945,10 @@
       <c r="B2" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D2" s="15" t="s">
+      <c r="D2" s="20" t="s">
         <v>52</v>
       </c>
       <c r="E2" s="2"/>
@@ -942,10 +960,10 @@
       <c r="B3" s="8" t="s">
         <v>47</v>
       </c>
-      <c r="C3" s="18" t="s">
+      <c r="C3" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="21" t="s">
         <v>52</v>
       </c>
       <c r="E3" s="1"/>
@@ -957,10 +975,10 @@
       <c r="B4" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="15" t="s">
+      <c r="D4" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E4" s="2"/>
@@ -972,10 +990,10 @@
       <c r="B5" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E5" s="1"/>
@@ -987,10 +1005,10 @@
       <c r="B6" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D6" s="15" t="s">
+      <c r="D6" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E6" s="2"/>
@@ -1002,10 +1020,10 @@
       <c r="B7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D7" s="15" t="s">
+      <c r="D7" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E7" s="1"/>
@@ -1017,10 +1035,10 @@
       <c r="B8" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D8" s="15" t="s">
+      <c r="D8" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E8" s="2"/>
@@ -1032,10 +1050,10 @@
       <c r="B9" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D9" s="15" t="s">
+      <c r="D9" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E9" s="1"/>
@@ -1047,215 +1065,230 @@
       <c r="B10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="20" t="s">
         <v>53</v>
       </c>
       <c r="E10" s="2"/>
     </row>
-    <row r="11" spans="1:5" ht="150" customHeight="1" x14ac:dyDescent="0.5">
+    <row r="11" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
       <c r="A11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>50</v>
+      </c>
+      <c r="D11" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E11" s="2"/>
+    </row>
+    <row r="12" spans="1:5" ht="150" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A12" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C12" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D12" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E12" s="1" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
-      <c r="A12" s="5" t="s">
+    <row r="13" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
+      <c r="A13" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="B12" s="11" t="s">
+      <c r="B13" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C13" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D13" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E12" s="2"/>
-    </row>
-    <row r="13" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
-      <c r="A13" s="3" t="s">
+      <c r="E13" s="2"/>
+    </row>
+    <row r="14" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
+      <c r="A14" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B14" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C14" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D14" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E13" s="1"/>
-    </row>
-    <row r="14" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
-      <c r="A14" s="2" t="s">
+      <c r="E14" s="1"/>
+    </row>
+    <row r="15" spans="1:5" ht="36.6" x14ac:dyDescent="0.5">
+      <c r="A15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="7" t="s">
+      <c r="B15" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C14" s="18" t="s">
+      <c r="C15" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D15" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E14" s="2"/>
-    </row>
-    <row r="15" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
-      <c r="A15" s="4" t="s">
+      <c r="E15" s="2"/>
+    </row>
+    <row r="16" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
+      <c r="A16" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B16" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="C15" s="18" t="s">
+      <c r="C16" s="15" t="s">
         <v>58</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D16" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E15" s="1"/>
-    </row>
-    <row r="16" spans="1:5" ht="37.799999999999997" x14ac:dyDescent="0.5">
-      <c r="A16" s="6" t="s">
+      <c r="E16" s="1"/>
+    </row>
+    <row r="17" spans="1:6" ht="37.799999999999997" x14ac:dyDescent="0.5">
+      <c r="A17" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B17" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="C16" s="18" t="s">
+      <c r="C17" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="E17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" ht="36.6" x14ac:dyDescent="0.5">
+      <c r="A18" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="B18" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="C18" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D18" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="2"/>
-    </row>
-    <row r="17" spans="1:6" ht="36.6" x14ac:dyDescent="0.5">
-      <c r="A17" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="B17" s="9" t="s">
-        <v>34</v>
-      </c>
-      <c r="C17" s="18" t="s">
+      <c r="E18" s="1"/>
+    </row>
+    <row r="19" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
+      <c r="A19" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D17" s="20" t="s">
-        <v>48</v>
-      </c>
-      <c r="E17" s="1"/>
-    </row>
-    <row r="18" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
-      <c r="A18" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="B18" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C18" s="18" t="s">
+      <c r="D19" s="22" t="s">
+        <v>52</v>
+      </c>
+      <c r="E19" s="2"/>
+    </row>
+    <row r="20" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
+      <c r="A20" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D18" s="17" t="s">
+      <c r="D20" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="E20" s="1"/>
+    </row>
+    <row r="21" spans="1:6" ht="54.6" x14ac:dyDescent="0.4">
+      <c r="A21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="C21" s="19" t="s">
+        <v>58</v>
+      </c>
+      <c r="D21" s="20" t="s">
+        <v>55</v>
+      </c>
+      <c r="E21" s="2"/>
+    </row>
+    <row r="22" spans="1:6" ht="72" x14ac:dyDescent="0.35">
+      <c r="A22" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B22" s="9" t="s">
+        <v>42</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D22" s="23" t="s">
         <v>52</v>
       </c>
-      <c r="E18" s="2"/>
-    </row>
-    <row r="19" spans="1:6" ht="36.6" x14ac:dyDescent="0.4">
-      <c r="A19" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="18" t="s">
+      <c r="E22" s="9"/>
+    </row>
+    <row r="23" spans="1:6" ht="54" x14ac:dyDescent="0.35">
+      <c r="A23" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="B23" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="C23" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="16" t="s">
+      <c r="D23" s="24" t="s">
+        <v>57</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" s="18" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" ht="82.2" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B24" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="C24" s="15" t="s">
+        <v>51</v>
+      </c>
+      <c r="D24" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E19" s="1"/>
-    </row>
-    <row r="20" spans="1:6" ht="54.6" x14ac:dyDescent="0.4">
-      <c r="A20" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="B20" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="C20" s="22" t="s">
-        <v>58</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>55</v>
-      </c>
-      <c r="E20" s="2"/>
-    </row>
-    <row r="21" spans="1:6" ht="72" x14ac:dyDescent="0.35">
-      <c r="A21" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="B21" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="C21" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="E21" s="9"/>
-    </row>
-    <row r="22" spans="1:6" ht="54" x14ac:dyDescent="0.35">
-      <c r="A22" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="B22" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="7" t="s">
-        <v>57</v>
-      </c>
-      <c r="E22" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="F22" s="21" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" ht="82.2" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A23" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B23" s="9" t="s">
-        <v>46</v>
-      </c>
-      <c r="C23" s="18" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="9"/>
+      <c r="E24" s="9"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:E1" xr:uid="{69A9896E-8EAC-4EAC-8BD0-8B557D602AA3}"/>
@@ -1271,7 +1304,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C23" xr:uid="{10875831-33C7-4878-9CE7-6731C744575D}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C24" xr:uid="{10875831-33C7-4878-9CE7-6731C744575D}">
       <formula1>"Pas commencé, En cours, Terminé"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
temp commit fo stash
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\Projet1_Jeux_Video\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chacy\My Shit\nbk\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0764F5B-01F9-4A21-89DA-7CF035D32C65}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87A82D4C-FBBE-489D-947F-D94CACF062F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="61">
   <si>
     <t>Fonctionnalites</t>
   </si>
@@ -314,7 +314,13 @@
     <t>tout le monde</t>
   </si>
   <si>
-    <t>Apparaît et bouge avec le joueur, reste à faire collisions</t>
+    <t>Reste a exploser quand entre en contact avec un enemi</t>
+  </si>
+  <si>
+    <t>Reste a exploser quand entre en contact avec un enemi + weird starting position</t>
+  </si>
+  <si>
+    <t>Reste a exploser quand entre en contact avec un enemi + finir seekEnemy</t>
   </si>
 </sst>
 </file>
@@ -992,7 +998,9 @@
       <c r="D6" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E6" s="22"/>
+      <c r="E6" s="22" t="s">
+        <v>60</v>
+      </c>
     </row>
     <row r="7" spans="1:5" ht="36" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
@@ -1039,7 +1047,9 @@
       <c r="D9" s="14" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="23"/>
+      <c r="E9" s="22" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="10" spans="1:5" ht="57" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">

</xml_diff>

<commit_message>
Animation de fin, Terminer.
</commit_message>
<xml_diff>
--- a/Taches.xlsx
+++ b/Taches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\travail\Projet1_Jeux_Video\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54303BC5-CC77-4A97-98B9-DF6BB0AE0827}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF827F62-3903-4769-B1CA-B4E8F740B6D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="0" windowWidth="21600" windowHeight="15585" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3BCE4F66-BD57-4DA1-9203-FCE236D7FCD6}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -281,98 +281,6 @@
   <si>
     <r>
       <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Au démarrage du jeu, le joueur est placé au centre et tout est figé jusqu’à ce qu’on appuie sur la touche espace.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>La partie commence alors.</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>La partie doit durer quelques minutes au plus et terminer si le joueur est éliminé</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="7"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>ou s’il élimine le boss</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>. Au moment que la partie se termine, détruire tous les ennemis et</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="14"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> figer le joueur en jouant l’animation appropriée.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <b/>
         <u/>
         <sz val="14"/>
@@ -558,6 +466,98 @@
       </rPr>
       <t xml:space="preserve">
 </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Au démarrage du jeu, le joueur est placé au centre et tout est figé jusqu’à ce qu’on appuie sur la touche espace.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>La partie commence alors.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>La partie doit durer quelques minutes au plus et terminer si le joueur est éliminé</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="7"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>ou s’il élimine le boss</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="14"/>
+        <color rgb="FF00B050"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Au moment que la partie se termine, détruire tous les ennemis et figer le joueur en jouant l’animation appropriée.</t>
     </r>
   </si>
 </sst>
@@ -1221,7 +1221,7 @@
         <v>5</v>
       </c>
       <c r="B3" s="7" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C3" s="16" t="s">
         <v>57</v>
@@ -1493,10 +1493,10 @@
         <v>40</v>
       </c>
       <c r="B21" s="8" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C21" s="16" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="D21" s="8" t="s">
         <v>49</v>

</xml_diff>